<commit_message>
#9 - 22/6 1
</commit_message>
<xml_diff>
--- a/frame.xlsx
+++ b/frame.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20730"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vay\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{734727AC-C2D5-4452-B495-C29A3CD68F05}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="45" windowWidth="27795" windowHeight="12600"/>
+    <workbookView xWindow="475" yWindow="41" windowWidth="27795" windowHeight="12607" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
   <si>
     <t>…</t>
   </si>
@@ -169,12 +175,33 @@
   </si>
   <si>
     <t>số trạng thái nhóm thứ N (byte cao)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">số lượng group trong project </t>
+  </si>
+  <si>
+    <t xml:space="preserve">id group thứ 0 </t>
+  </si>
+  <si>
+    <t>số trạng thái của group thứ 0 (byte thấp)</t>
+  </si>
+  <si>
+    <t>số trạng thái của group thứ 0 (byte cao)</t>
+  </si>
+  <si>
+    <t>thời gian trạng thái 0 của group thứ 0</t>
+  </si>
+  <si>
+    <t>… thời gian trạn thái n của group thứ 0</t>
+  </si>
+  <si>
+    <t>… id group thứ N</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -442,7 +469,7 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -514,6 +541,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -521,6 +551,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="8" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -539,6 +572,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -587,7 +623,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -620,9 +656,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -655,6 +708,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -830,21 +900,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="64.28515625" customWidth="1"/>
+    <col min="1" max="1" width="64.25" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="73.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" customWidth="1"/>
-    <col min="6" max="6" width="39.140625" customWidth="1"/>
-    <col min="7" max="7" width="58.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="48.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="73.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.25" customWidth="1"/>
+    <col min="6" max="6" width="39.125" customWidth="1"/>
+    <col min="7" max="7" width="58.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="48.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="27.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>9</v>
       </c>
@@ -860,7 +930,7 @@
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
-      <c r="H1" s="42" t="s">
+      <c r="H1" s="43" t="s">
         <v>10</v>
       </c>
     </row>
@@ -884,13 +954,13 @@
       <c r="G2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="42"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="40">
+      <c r="B3" s="41">
         <v>4</v>
       </c>
       <c r="C3" s="20"/>
@@ -902,12 +972,12 @@
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="42"/>
+      <c r="H3" s="43"/>
       <c r="I3" s="15"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
-      <c r="B4" s="40"/>
+      <c r="B4" s="41"/>
       <c r="C4" s="20"/>
       <c r="D4" s="2" t="s">
         <v>2</v>
@@ -917,12 +987,12 @@
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="42"/>
+      <c r="H4" s="43"/>
       <c r="I4" s="15"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
-      <c r="B5" s="40"/>
+      <c r="B5" s="41"/>
       <c r="C5" s="21"/>
       <c r="D5" s="22" t="s">
         <v>3</v>
@@ -932,14 +1002,14 @@
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="42"/>
+      <c r="H5" s="43"/>
       <c r="I5" s="15"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="40"/>
+      <c r="B6" s="41"/>
       <c r="C6" s="21"/>
       <c r="D6" s="2" t="s">
         <v>21</v>
@@ -949,7 +1019,7 @@
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
-      <c r="H6" s="42"/>
+      <c r="H6" s="43"/>
       <c r="I6" s="15"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -962,13 +1032,13 @@
       <c r="E7" s="23"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="42"/>
+      <c r="H7" s="43"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="40">
+      <c r="B8" s="41">
         <v>4</v>
       </c>
       <c r="C8" s="21"/>
@@ -976,12 +1046,12 @@
       <c r="E8" s="23"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="42"/>
+      <c r="H8" s="43"/>
       <c r="I8" s="15"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="6"/>
-      <c r="B9" s="40"/>
+      <c r="B9" s="41"/>
       <c r="C9" s="21"/>
       <c r="D9" s="3" t="s">
         <v>23</v>
@@ -989,12 +1059,12 @@
       <c r="E9" s="23"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="42"/>
+      <c r="H9" s="43"/>
       <c r="I9" s="15"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="40"/>
+      <c r="B10" s="41"/>
       <c r="C10" s="21"/>
       <c r="D10" s="3" t="s">
         <v>24</v>
@@ -1002,24 +1072,24 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
-      <c r="H10" s="42"/>
+      <c r="H10" s="43"/>
       <c r="I10" s="15"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="40"/>
+      <c r="B11" s="41"/>
       <c r="C11" s="24"/>
       <c r="D11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="41">
+      <c r="E11" s="42">
         <v>4</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
-      <c r="H11" s="42"/>
+      <c r="H11" s="43"/>
       <c r="I11" s="15"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1028,39 +1098,45 @@
       </c>
       <c r="C12" s="24"/>
       <c r="D12" s="2"/>
-      <c r="E12" s="41"/>
+      <c r="E12" s="42"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="42"/>
+      <c r="H12" s="43"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>11</v>
+        <v>51</v>
       </c>
       <c r="C13" s="24"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="41"/>
+      <c r="E13" s="42"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
-      <c r="H13" s="42"/>
+      <c r="H13" s="43"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="5"/>
+        <v>52</v>
+      </c>
+      <c r="B14" s="40">
+        <v>1</v>
+      </c>
       <c r="C14" s="24"/>
       <c r="D14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="41"/>
+      <c r="E14" s="42"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
-      <c r="H14" s="42"/>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
+      <c r="H14" s="43"/>
+    </row>
+    <row r="15" spans="1:9" ht="14.95" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="45">
+        <v>2</v>
+      </c>
       <c r="C15" s="24"/>
       <c r="D15" s="2" t="s">
         <v>27</v>
@@ -1068,11 +1144,13 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="42"/>
-    </row>
-    <row r="16" spans="1:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
+      <c r="H15" s="43"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.65" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="45"/>
       <c r="C16" s="13" t="s">
         <v>28</v>
       </c>
@@ -1086,11 +1164,15 @@
         <v>6</v>
       </c>
       <c r="G16" s="28"/>
-      <c r="H16" s="42"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
+      <c r="H16" s="43"/>
+    </row>
+    <row r="17" spans="1:8" ht="14.95" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
       <c r="C17" s="24"/>
       <c r="D17" s="7" t="s">
         <v>30</v>
@@ -1100,10 +1182,12 @@
       </c>
       <c r="F17" s="24"/>
       <c r="G17" s="29"/>
-      <c r="H17" s="42"/>
+      <c r="H17" s="43"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
+      <c r="A18" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="B18" s="1"/>
       <c r="C18" s="21"/>
       <c r="D18" s="8" t="s">
@@ -1112,10 +1196,12 @@
       <c r="E18" s="30"/>
       <c r="F18" s="24"/>
       <c r="G18" s="29"/>
-      <c r="H18" s="42"/>
+      <c r="H18" s="43"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
+      <c r="A19" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="B19" s="1"/>
       <c r="C19" s="21"/>
       <c r="D19" s="9" t="s">
@@ -1126,10 +1212,12 @@
       </c>
       <c r="F19" s="24"/>
       <c r="G19" s="29"/>
-      <c r="H19" s="42"/>
+      <c r="H19" s="43"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
+      <c r="A20" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B20" s="1"/>
       <c r="C20" s="21"/>
       <c r="D20" s="9" t="s">
@@ -1138,10 +1226,12 @@
       <c r="E20" s="31"/>
       <c r="F20" s="24"/>
       <c r="G20" s="29"/>
-      <c r="H20" s="42"/>
+      <c r="H20" s="43"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
+      <c r="A21" s="6" t="s">
+        <v>11</v>
+      </c>
       <c r="B21" s="1"/>
       <c r="C21" s="20"/>
       <c r="D21" s="10" t="s">
@@ -1152,10 +1242,12 @@
       </c>
       <c r="F21" s="24"/>
       <c r="G21" s="29"/>
-      <c r="H21" s="42"/>
+      <c r="H21" s="43"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
+      <c r="A22" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="C22" s="20"/>
       <c r="D22" s="32" t="s">
         <v>35</v>
@@ -1165,7 +1257,7 @@
       </c>
       <c r="F22" s="24"/>
       <c r="G22" s="29"/>
-      <c r="H22" s="42"/>
+      <c r="H22" s="43"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C23" s="20"/>
@@ -1177,7 +1269,7 @@
       </c>
       <c r="F23" s="24"/>
       <c r="G23" s="29"/>
-      <c r="H23" s="42"/>
+      <c r="H23" s="43"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C24" s="20"/>
@@ -1189,7 +1281,7 @@
       </c>
       <c r="F24" s="24"/>
       <c r="G24" s="29"/>
-      <c r="H24" s="42"/>
+      <c r="H24" s="43"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C25" s="20"/>
@@ -1199,7 +1291,7 @@
       <c r="E25" s="31"/>
       <c r="F25" s="24"/>
       <c r="G25" s="29"/>
-      <c r="H25" s="42"/>
+      <c r="H25" s="43"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C26" s="20"/>
@@ -1211,7 +1303,7 @@
       </c>
       <c r="F26" s="24"/>
       <c r="G26" s="29"/>
-      <c r="H26" s="42"/>
+      <c r="H26" s="43"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C27" s="24"/>
@@ -1221,7 +1313,7 @@
       <c r="E27" s="31"/>
       <c r="F27" s="24"/>
       <c r="G27" s="29"/>
-      <c r="H27" s="42"/>
+      <c r="H27" s="43"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C28" s="24"/>
@@ -1231,7 +1323,7 @@
       <c r="E28" s="31"/>
       <c r="F28" s="24"/>
       <c r="G28" s="29"/>
-      <c r="H28" s="42"/>
+      <c r="H28" s="43"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B29" s="5"/>
@@ -1244,7 +1336,7 @@
       </c>
       <c r="F29" s="24"/>
       <c r="G29" s="29"/>
-      <c r="H29" s="42"/>
+      <c r="H29" s="43"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B30" s="5"/>
@@ -1257,7 +1349,7 @@
       </c>
       <c r="F30" s="24"/>
       <c r="G30" s="29"/>
-      <c r="H30" s="42"/>
+      <c r="H30" s="43"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C31" s="24"/>
@@ -1269,7 +1361,7 @@
       </c>
       <c r="F31" s="24"/>
       <c r="G31" s="29"/>
-      <c r="H31" s="42"/>
+      <c r="H31" s="43"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C32" s="24"/>
@@ -1279,9 +1371,9 @@
       <c r="E32" s="31"/>
       <c r="F32" s="24"/>
       <c r="G32" s="29"/>
-      <c r="H32" s="42"/>
-    </row>
-    <row r="33" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H32" s="43"/>
+    </row>
+    <row r="33" spans="2:8" ht="14.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C33" s="24"/>
       <c r="D33" s="9" t="s">
         <v>45</v>
@@ -1291,9 +1383,9 @@
       </c>
       <c r="F33" s="24"/>
       <c r="G33" s="29"/>
-      <c r="H33" s="42"/>
-    </row>
-    <row r="34" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H33" s="43"/>
+    </row>
+    <row r="34" spans="2:8" ht="14.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="24"/>
       <c r="D34" s="12" t="s">
         <v>46</v>
@@ -1301,9 +1393,9 @@
       <c r="E34" s="33"/>
       <c r="F34" s="34"/>
       <c r="G34" s="35"/>
-      <c r="H34" s="42"/>
-    </row>
-    <row r="35" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H34" s="43"/>
+    </row>
+    <row r="35" spans="2:8" ht="14.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C35" s="21"/>
       <c r="D35" s="6" t="s">
         <v>7</v>
@@ -1311,9 +1403,9 @@
       <c r="E35" s="2"/>
       <c r="F35" s="36"/>
       <c r="G35" s="36"/>
-      <c r="H35" s="42"/>
-    </row>
-    <row r="36" spans="2:8" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H35" s="43"/>
+    </row>
+    <row r="36" spans="2:8" ht="14.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C36" s="21" t="s">
         <v>47</v>
       </c>
@@ -1323,9 +1415,9 @@
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
-      <c r="H36" s="42"/>
-    </row>
-    <row r="37" spans="2:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="H36" s="43"/>
+    </row>
+    <row r="37" spans="2:8" ht="14.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C37" s="21"/>
       <c r="D37" s="4" t="s">
         <v>49</v>
@@ -1333,9 +1425,9 @@
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
-      <c r="H37" s="42"/>
-    </row>
-    <row r="38" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H37" s="43"/>
+    </row>
+    <row r="38" spans="2:8" ht="21.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="24"/>
       <c r="D38" s="4" t="s">
         <v>50</v>
@@ -1343,7 +1435,7 @@
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
-      <c r="H38" s="42"/>
+      <c r="H38" s="43"/>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C39" s="37"/>
@@ -1353,9 +1445,9 @@
       <c r="E39" s="39"/>
       <c r="F39" s="39"/>
       <c r="G39" s="39"/>
-      <c r="H39" s="43"/>
-    </row>
-    <row r="40" spans="2:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="H39" s="44"/>
+    </row>
+    <row r="40" spans="2:8" ht="21.1" x14ac:dyDescent="0.25">
       <c r="B40" s="5"/>
       <c r="C40" s="17"/>
       <c r="D40" s="17"/>
@@ -1363,7 +1455,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="2:8" ht="21" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:8" ht="21.1" x14ac:dyDescent="0.25">
       <c r="C41" s="17"/>
       <c r="D41" s="17"/>
       <c r="E41" s="17"/>
@@ -1383,11 +1475,12 @@
       <c r="C45" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="B3:B6"/>
     <mergeCell ref="B8:B11"/>
     <mergeCell ref="E11:E14"/>
     <mergeCell ref="H1:H39"/>
+    <mergeCell ref="B15:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="256" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
@@ -1395,18 +1488,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>